<commit_message>
chore(publish): 刷新更新时间与下载文件 2026-09-13 18:09
</commit_message>
<xml_diff>
--- a/dataset/全国重点院校/全国高校汇总表.xlsx
+++ b/dataset/全国重点院校/全国高校汇总表.xlsx
@@ -201,8 +201,7 @@
 智能交互学院 | https://sii.ecnu.edu.cn/ | 电话:009102000042
 上海国际首席技术官学院 | https://cto.ecnu.edu.cn/main.htm | 电话:021-61911352
 精密光谱科学与技术高等研究院 | http://www.lps.ecnu.edu.cn/ | 邮箱:lps@phy.ecnu.edu.cn | 电话:021-54836023
-量子科学与精密测量研究院 | https://iqspm.ecnu.edu.cn/index.html?_refluxos=a10https://iqspm.ecnu.edu.cn/index.html?_refluxos=a10 | 邮箱:jtsheng@lps.ecnu.edu.cn | 电话:(86)21-54836079
-地理科学学院 | http://www.geo.ecnu.edu.cn/ | 邮箱:ghwang@geo.ec; geo@geo.ecnu.edu.cn | 电话:54341218</t>
+量子科学与精密测量研究院 | https://iqspm.ecnu.edu.cn/index.html?_refluxos=a10https://iqspm.ecnu.edu.cn/index.html?_refluxos=a10 | 邮箱:jtsheng@lps.ecnu.edu.cn | 电话:(86)21-54836079</t>
   </si>
   <si>
     <t>同济大学</t>
@@ -300,7 +299,7 @@
     <t>数学科学学院 | http://math.fudan.edu.cn/ | 邮箱:sxbks@fudan.edu.cn | 电话:021-65642222; 55665146）; 65643503）
 微电子学院 | https://sme.fudan.edu.cn/ | 邮箱:sme_keyan@fudan.edu.cn; sme_admission@fudan.edu.cn; sme@fudan.edu.cn | 电话:021-65641106; 021-65643449; 021-65643438
 生命科学学院 | http://life.fudan.edu.cn/ | 电话:08660525549
-大数据学院 | http://www.sds.fudan.edu.cn/wp/
+大数据学院 | https://sds.fudan.edu.cn/
 集成电路与微纳电子创新学院 | https://icmne.fudan.edu.cn/ | 邮箱:icmne@fudan.edu.cn
 计算与智能创新学院 | https://ai.fudan.edu.cn/ | 邮箱:cs_school@fudan.edu.cn | 电话:13472188450
 智能机器人与先进制造创新学院 | https://ciram.fudan.edu.cn/ | 邮箱:ciram_dzb@fudan.edu.cn; yingsun@fudan.edu.cn; teai@fudan.edu.cn | 电话:021-65641208; 021-31243536; 021-65642740
@@ -324,18 +323,18 @@
     <t>https://pgs.ruc.edu.cn/gats.htm</t>
   </si>
   <si>
-    <t>■ 生态环境学院 | https://envi.ruc.edu.cn/ | 邮箱:huanjing@ruc.edu.cn | 电话:010-62511042
-■ 信息学院 | http://info.ruc.edu.cn/
-■ 统计学院 | http://stat.ruc.edu.cn/ | 邮箱:tongjioffice@ruc.edu.cn | 电话:01620241114; 010-62511318; 010-62511316
-■ 化学与生命资源学院 | https://clr.ruc.edu.cn/zwwz/index.htm | 邮箱:ruc_clr@ruc.edu.cn | 电话:010-62512822
-■ 物理学院 | http://www.phys.ruc.edu.cn/ | 邮箱:graphy@ruc.edu.cn | 电话:+86-10-62517997（
-■ 统计与大数据研究院 | http://isbd.ruc.edu.cn/
-■ 数学学院 | http://math.ruc.edu.cn/ | 邮箱:mathruc@ruc.edu.cn | 电话:010-82507161
-■ 高瓴人工智能学院 | http://ai.ruc.edu.cn/ | 邮箱:ai@ruc.edu.cn
-■ 智慧治理学院 | http://su.ruc.edu.cn/department/ssg/index.htm | 电话:045931565425
+    <t>生态环境学院 | https://envi.ruc.edu.cn/ | 邮箱:huanjing@ruc.edu.cn | 电话:010-62511042
+信息学院 | http://info.ruc.edu.cn/
+统计学院 | http://stat.ruc.edu.cn/ | 邮箱:tongjioffice@ruc.edu.cn | 电话:01620241114; 010-62511318; 010-62511316
+化学与生命资源学院 | https://clr.ruc.edu.cn/zwwz/index.htm | 邮箱:ruc_clr@ruc.edu.cn | 电话:010-62512822
+物理学院 | http://www.phys.ruc.edu.cn/ | 邮箱:graphy@ruc.edu.cn | 电话:+86-10-62517997（
+统计与大数据研究院 | http://isbd.ruc.edu.cn/
+数学学院 | http://math.ruc.edu.cn/ | 邮箱:mathruc@ruc.edu.cn | 电话:010-82507161
+高瓴人工智能学院 | http://ai.ruc.edu.cn/ | 邮箱:ai@ruc.edu.cn
+智慧治理学院 | http://su.ruc.edu.cn/department/ssg/index.htm | 电话:045931565425
 国家治理工程学院 | http://ang.ruc.edu.cn/index.htm | 邮箱:GJZL@ruc.edu.cn | 电话:010-62510553
-■ 全球领导力学院 | http://sgl.ruc.edu.cn/ | 邮箱:sglruc@ruc.edu.cn
-■ 交叉科学研究院 | http://sids.ruc.edu.cn/ | 邮箱:rdcy2021@ruc.edu.cn | 电话:010-62510183</t>
+全球领导力学院 | http://sgl.ruc.edu.cn/ | 邮箱:sglruc@ruc.edu.cn
+交叉科学研究院 | http://sids.ruc.edu.cn/ | 邮箱:rdcy2021@ruc.edu.cn | 电话:010-62510183</t>
   </si>
   <si>
     <t>中国农业大学</t>
@@ -615,8 +614,7 @@
 交叉信息研究院 | https://iiis.tsinghua.edu.cn/ | 邮箱:iiis@mail.tsinghua.edu.cn | 电话:010-62781693
 航空发动机研究院 | http://www.ae.tsinghua.edu.cn/ | 邮箱:hfyzhb@mailoa.tsinghua.edu.cn; hfykyb@tsinghua.edu.cn | 电话:62796693; 62786853; 62771763
 智能产业研究院 | https://air.tsinghua.edu.cn/ | 邮箱:airoffice@air.tsinghua.edu.cn; airhr@air.tsinghua.edu.cn | 电话:(010)82151160
-国家卓越工程师学院 | https://www.ngce.tsinghua.edu.cn/ | 邮箱:gcsxy@tsinghua.edu.cn | 电话:010-62793784
-人工智能学院 | http://collegeai.tsinghua.edu.cn/ | 邮箱:collegeai@mail.tsinghua.edu.cn | 电话:62788817</t>
+国家卓越工程师学院 | https://www.ngce.tsinghua.edu.cn/ | 邮箱:gcsxy@tsinghua.edu.cn | 电话:010-62793784</t>
   </si>
   <si>
     <t>吉林省</t>
@@ -1316,26 +1314,26 @@
     <t>科学技术研究院 | http://rd.zju.edu.cn/
 技术转化研究院 | http://www.itt.zju.edu.cn/ | 邮箱:lwu@zju.edu.cn; quxiaodi@zju.edu.cn; ltm@zju.edu.cn | 电话:0571-88982935
 数学科学学院
-物理学院
+物理学院 | https://physics.zju.edu.cn/
 地球科学学院
-机械工程学院
-材料科学与工程学院
+机械工程学院 | http://me.zju.edu.cn/
+材料科学与工程学院 | https://mse.zju.edu.cn/
 能源工程学院
-电气工程学院
+电气工程学院 | http://ee.zju.edu.cn/
 建筑工程学院
-化学工程与生物工程学院
-海洋学院
-航空航天学院
-光电科学与工程学院
+化学工程与生物工程学院 | http://che.zju.edu.cn/
+海洋学院 | http://oc.zju.edu.cn/
+航空航天学院 | http://saa.zju.edu.cn/
+光电科学与工程学院 | http://opt.zju.edu.cn/
 信息与电子工程学院
-控制科学与工程学院
+控制科学与工程学院 | http://cse.zju.edu.cn/
 计算机科学与技术学院 —网络空间安全学院
 计算机科学与技术学院
-—网络空间安全学院
+网络空间安全学院
 软件学院
 生物医学工程与仪器科学学院
-集成电路学院
-人工智能学院
+集成电路学院 | https://ic.zju.edu.cn/
+人工智能学院 | https://ai.zju.edu.cn/
 生命科学学院
 生物系统工程与食品科学学院
 环境与资源学院
@@ -1750,7 +1748,7 @@
 材料科学与工程学院 | http://mse.dlut.edu.cn | 邮箱:mse@dlut.edu.cn | 电话:0411-84708430
 能源与动力学院 | http://power.dlut.edu.cn | 邮箱:powere@dlut.edu.cn | 电话:0411-84708460
 电子信息与电气工程学部 | http://ee.dlut.edu.cn/ | 邮箱:dutee@dlut.edu.cn | 电话:0411-84706936
-电气工程学院 | http://eee.dlut.edu.cn
+电气工程学院 | https://ee.dlut.edu.cn/
 信息与通信工程学院 | http://ice.dlut.edu.cn | 邮箱:bowang@dlut.edu.cn
 控制科学与工程学院 | http://scse.dlut.edu.cn | 邮箱:cse@dlut.edu.cn | 电话:0411-84701537
 计算机科学与技术学院 | http://cs.dlut.edu.cn
@@ -2212,8 +2210,7 @@
   </si>
   <si>
     <t>华东化工学院 | https://www.ecust.edu.cn/847/list.htm | 电话:009102000037
-上海化工学院 | https://www.ecust.edu.cn/shhgxy/list.htm | 电话:009102000037
-华东化工学院 | https://www.ecust.edu.cn/709/list.htm | 电话:009102000037</t>
+上海化工学院 | https://www.ecust.edu.cn/shhgxy/list.htm | 电话:009102000037</t>
   </si>
   <si>
     <t>第二军医大学</t>
@@ -2431,13 +2428,7 @@
 人工智能学院 | https://ai.cumtb.edu.cn/ | 邮箱:rgznxy@cumtb.edu.cn | 电话:010-62339761
 力学与土木工程学院 | http://ljxy.cumtb.edu.cn/
 理学院 | http://lxy.cumtb.edu.cn/
-中国矿业大学（北京）内蒙古研究院 | https://nmgyjy.cumtb.edu.cn/ | 电话:17854205908
-能源与矿业学院 | https://nyxy.cumtb.edu.cn
-地球科学与测绘工程学院 | https://dcxy.cumtb.edu.cn/ | 邮箱:yzxxdcxy@163.com | 电话:010-62339300
-化学与环境工程学院 | https://scee.cumtb.edu.cn/
-机械与电气工程学院 | https://jdxy.cumtb.edu.cn/ | 邮箱:jdxy@cumtb.edu.cn | 电话:010-62331370
-力学与土木工程学院 | https://ljxy.cumtb.edu.cn/
-理学院 | https://lxy.cumtb.edu.cn/</t>
+中国矿业大学（北京）内蒙古研究院 | https://nmgyjy.cumtb.edu.cn/ | 电话:17854205908</t>
   </si>
   <si>
     <t>中央财经大学</t>
@@ -2759,8 +2750,7 @@
 工程技术研究院 | http://iet.ustb.edu.cn/ | 邮箱:bkdgyy@ustb.edu.cn | 电话:010-62332598
 大安全科学研究院 | https://mss.ustb.edu.cn/ | 电话:010-62333808
 城镇化与城市安全研究院 | https://iuus.ustb.edu.cn | 电话:010-62334196
-科学技术研究院 | https://research.ustb.edu.cn/ | 电话:0402430062
-资源与安全工程学院 | http://cres.ustb.edu.cn/</t>
+科学技术研究院 | https://research.ustb.edu.cn/ | 电话:0402430062</t>
   </si>
   <si>
     <t>北京邮电大学</t>
@@ -3954,22 +3944,6 @@
 环境科学与工程学院 | http://sese.hainanu.edu.cn | 电话:0898-66255157
 食品科学与工程学院 | https://hd.hainanu.edu.cn/shipin/
 海洋生物与水产学院 | http://smbf.hainanu.edu.cn | 邮箱:xiesg@hainanu.edu.cn; 993928@hainanu.edu.cn; haiyyb@hainu.edu.cn | 电话:0898-66279184
-空天智能学院 | https://sai.hainanu.edu.cn/ | 邮箱:ktzn@hainanu.edu.cn | 电话:0898-66268297
-数学与统计学院 | http://sms.hainanu.edu.cn | 邮箱:hdsxtj@hainanu.edu.cn
-物理与光电工程学院 | http://spoe.hainanu.edu.cn | 邮箱:wdxyzh@hainanu.edu.cn | 电话:0898-66279161
-化学化工学院 | http://scce.hainanu.edu.cn | 邮箱:hdhg@hainanu.edu.cn | 电话:0898-66255906; 0898-66256050; 0898-66279224
-生命健康学院 | http://slhs.hainanu.edu.cn | 邮箱:hdsmkx@hainanu.edu.cn | 电话:0898-66253203（
-机电工程学院 | http://smee.hainanu.edu.cn | 电话:0898-66267576; 0898-66271526; 0898-66267372
-材料科学与工程学院 | http://mse.hainanu.edu.cn | 邮箱:clxyzhb@hainanu.edu.cn | 电话:0898-66251982（
-电子科学与技术学院 | https://hd.hainanu.edu.cn/dzkx/
-信息与通信工程学院 | http://sice.hainanu.edu.cn | 邮箱:sice@hainan.edu.cn | 电话:0898-66279057
-计算机科学与技术学院 | http://cs.hainanu.edu.cn | 邮箱:cs@hainanu.edu.cn | 电话:0898-66278203
-网络空间安全学院 | https://scs.hainanu.edu.cn/ | 邮箱:scscs@hainanu.edu.cn | 电话:0898-66259127; 0898-66257132
-土木建筑工程学院 | http://scea.hainanu.edu.cn | 电话:0898-66279232
-海洋技术与装备学院 | http://smse.hainanu.edu.cn/ | 邮箱:sheny2000@hainanu.edu.cn; 991302@hainanu.edu.cn | 电话:0898-66192572; 0898-66255276
-环境科学与工程学院 | http://sese.hainanu.edu.cn | 电话:0898-66255157
-食品科学与工程学院 | https://hd.hainanu.edu.cn/shipin/
-海洋生物与水产学院 | http://smbf.hainanu.edu.cn | 邮箱:xiesg@hainanu.edu.cn; 993928@hainanu.edu.cn; haiyyb@hainu.edu.cn | 电话:0898-66279184
 空天智能学院 | https://sai.hainanu.edu.cn/ | 邮箱:ktzn@hainanu.edu.cn | 电话:0898-66268297</t>
   </si>
   <si>
@@ -4122,13 +4096,13 @@
 等共计 助理</t>
   </si>
   <si>
-    <t>◆ 心理学院 | http://psych.ccnu.edu.cn/ | 电话:027-67868680
-◆ 数学与统计学学院 | http://maths.ccnu.edu.cn/
-◆ 物理科学与技术学院 | http://phy.ccnu.edu.cn/ | 电话:027-67867017
-◆ 化学学院 | http://chem.ccnu.edu.cn/ | 电话:027-67867955
-◆ 生命科学学院 | http://bio.ccnu.edu.cn/ | 电话:+86-27-67867221
-◆ 计算机学院 | http://cs.ccnu.edu.cn/ | 邮箱:cs@ccnu.edu.cn | 电话:027-67868318
-◆ 城市与环境科学学院 | http://ccnucity.ccnu.edu.cn/ | 电话:027-67868305; 027-67861443; 027-67867610</t>
+    <t>心理学院 | http://psych.ccnu.edu.cn/ | 电话:027-67868680
+数学与统计学学院 | http://maths.ccnu.edu.cn/
+物理科学与技术学院 | http://phy.ccnu.edu.cn/ | 电话:027-67867017
+化学学院 | http://chem.ccnu.edu.cn/ | 电话:027-67867955
+生命科学学院 | http://bio.ccnu.edu.cn/ | 电话:+86-27-67867221
+计算机学院 | http://cs.ccnu.edu.cn/ | 邮箱:cs@ccnu.edu.cn | 电话:027-67868318
+城市与环境科学学院 | http://ccnucity.ccnu.edu.cn/ | 电话:027-67868305; 027-67861443; 027-67867610</t>
   </si>
   <si>
     <t>武汉理工大学</t>
@@ -4215,13 +4189,6 @@
   </si>
   <si>
     <t>地理科学学院 | http://dlkx.hunnu.edu.cn/ | 邮箱:zhxy@hunnu.edu.cn | 电话:0731-88872535
-国际汉语文化学院 | http://icclc.hunnu.edu.cn/ | 邮箱:icclc@hunnu.edu.cn | 电话:0731-88873017
-化学化工学院 | http://hgxy.hunnu.edu.cn/ | 电话:88872530
-生命科学学院 | http://lifescience.hunnu.edu.cn/ | 电话:18890054350); 0731-88872525
-数学与统计学院 | http://mc.hunnu.edu.cn/ | 电话:0731-88872515
-物理与电子科学学院 | http://wdy.hunnu.edu.cn | 邮箱:wdy@hunnu.edu.cn | 电话:0731-88872520
-信息科学与工程学院 | http://cise.hunnu.edu.cn | 邮箱:641381226@qq.com
-地理科学学院 | http://dlkx.hunnu.edu.cn/ | 邮箱:zhxy@hunnu.edu.cn | 电话:0731-88872535
 国际汉语文化学院 | http://icclc.hunnu.edu.cn/ | 邮箱:icclc@hunnu.edu.cn | 电话:0731-88873017
 化学化工学院 | http://hgxy.hunnu.edu.cn/ | 电话:88872530
 生命科学学院 | http://lifescience.hunnu.edu.cn/ | 电话:18890054350); 0731-88872525
@@ -6312,18 +6279,6 @@
 计算机与软件学院 | http://csse.szu.edu.cn/
 人工智能学院 | https://ai.szu.edu.cn/ | 电话:0755-26946884
 建筑与城市规划学院 | http://saup.szu.edu.cn/ | 电话:(0755)26732877; (0755)26536114
-土木与交通工程学院 | http://ce.szu.edu.cn/ | 电话:（0755）26735711
-心理学院 | http://psy.szu.edu.cn/ | 邮箱:psych@szu.edu.cn | 电话:075526917503
-数学科学学院 | http://math.szu.edu.cn/ | 电话:0755-26534791
-物理与光电工程学院 | http://cpoe.szu.edu.cn/ | 邮箱:cpoe@szu.edu.cn | 电话:0755-26538735
-化学与环境工程学院 | http://chem.szu.edu.cn/ | 电话:0755-26536141
-生命与海洋科学学院 | http://bio.szu.edu.cn/ | 邮箱:szsky@szu.edu.cn | 电话:0755-86713951
-机电与控制工程学院 | http://cmce.szu.edu.cn/ | 电话:0755-26536224
-材料学院 | http://cmse.szu.edu.cn/ | 邮箱:guoyanke@szu.edu.cn
-电子与信息工程学院 | http://ceie.szu.edu.cn/ | 邮箱:cie@szu.edu.cn | 电话:0755-26536198
-计算机与软件学院 | http://csse.szu.edu.cn/
-人工智能学院 | https://ai.szu.edu.cn/ | 电话:0755-26946884
-建筑与城市规划学院 | http://saup.szu.edu.cn/ | 电话:(0755)26732877; (0755)26536114
 土木与交通工程学院 | http://ce.szu.edu.cn/ | 电话:（0755）26735711</t>
   </si>
   <si>
@@ -6912,13 +6867,6 @@
 电气与电子工程学院 | http://eee.wzu.edu.cn/ | 邮箱:dqdzxy@wzu.edu.cn | 电话:0577-86689010
 计算机与人工智能学院 | http://ai.wzu.edu.cn/ | 邮箱:ai@wzu.edu.cn | 电话:0577-86599385; 0577-86590231; 0577-86599563
 建筑工程学院 | http://cace.wzu.edu.cn/ | 邮箱:wzjgxy@wzu.edu.cn | 电话:0577-86689611
-数理学院 | https://slxy.wzu.edu.cn/ | 邮箱:slxy@wzu.edu.cn | 电话:0577-86689098; 0577-86689528
-化学与材料工程学院 | https://chem.wzu.edu.cn/ | 邮箱:hxx@wzu.edu.cn | 电话:0577-86689360; 0577-86689300; 0577-86689302
-生命与环境科学学院 | https://shxy.wzu.edu.cn/
-机电工程学院 | https://jdxy.wzu.edu.cn/
-电气与电子工程学院 | https://eee.wzu.edu.cn/ | 邮箱:dqdzxy@wzu.edu.cn | 电话:0577-86689010
-计算机与人工智能学院 | https://ai.wzu.edu.cn/ | 邮箱:ai@wzu.edu.cn | 电话:0577-86599385; 0577-86590231; 0577-86599563
-建筑工程学院 | https://cace.wzu.edu.cn/ | 邮箱:wzjgxy@wzu.edu.cn | 电话:0577-86689611
 新材料与产业技术研究院 | https://inmit.wzu.edu.cn/ | 邮箱:wzumit@163.com | 电话:0577-85516217
 激光与光电智能制造研究院 | https://im.wzu.edu.cn | 邮箱:imlp@wzu.edu.cn | 电话:0577-85516755</t>
   </si>
@@ -7984,7 +7932,7 @@
         <v>26</v>
       </c>
       <c r="U4" s="3">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="V4" s="3" t="s">
         <v>45</v>
@@ -8694,7 +8642,7 @@
         <v>121</v>
       </c>
       <c r="U14" s="3">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="V14" s="3" t="s">
         <v>124</v>
@@ -10966,7 +10914,7 @@
         <v>26</v>
       </c>
       <c r="U46" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V46" s="4" t="s">
         <v>430</v>
@@ -11534,7 +11482,7 @@
         <v>26</v>
       </c>
       <c r="U54" s="4">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="V54" s="4" t="s">
         <v>486</v>
@@ -12244,7 +12192,7 @@
         <v>26</v>
       </c>
       <c r="U64" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="V64" s="4" t="s">
         <v>559</v>
@@ -14516,7 +14464,7 @@
         <v>26</v>
       </c>
       <c r="U96" s="4">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="V96" s="4" t="s">
         <v>817</v>
@@ -14942,7 +14890,7 @@
         <v>26</v>
       </c>
       <c r="U102" s="4">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="V102" s="4" t="s">
         <v>870</v>
@@ -19273,7 +19221,7 @@
         <v>1346</v>
       </c>
       <c r="U163" s="6">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="V163" s="6" t="s">
         <v>1347</v>
@@ -20480,7 +20428,7 @@
         <v>26</v>
       </c>
       <c r="U180" s="6">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="V180" s="6" t="s">
         <v>1492</v>

</xml_diff>

<commit_message>
chore(publish): 刷新更新时间与下载文件 2026-09-15 14:04
</commit_message>
<xml_diff>
--- a/dataset/全国重点院校/全国高校汇总表.xlsx
+++ b/dataset/全国重点院校/全国高校汇总表.xlsx
@@ -3930,14 +3930,14 @@
 生命健康学院 | http://slhs.hainanu.edu.cn | 邮箱:hdsmkx@hainanu.edu.cn | 电话:0898-66253203（
 机电工程学院 | http://smee.hainanu.edu.cn | 电话:0898-66267576; 0898-66271526; 0898-66267372
 材料科学与工程学院 | http://mse.hainanu.edu.cn | 邮箱:clxyzhb@hainanu.edu.cn | 电话:0898-66251982（
-电子科学与技术学院 | https://hd.hainanu.edu.cn/dzkx/
+电子科学与技术学院 | https://ee.hainanu.edu.cn
 信息与通信工程学院 | http://sice.hainanu.edu.cn | 邮箱:sice@hainan.edu.cn | 电话:0898-66279057
 计算机科学与技术学院 | http://cs.hainanu.edu.cn | 邮箱:cs@hainanu.edu.cn | 电话:0898-66278203
 网络空间安全学院 | https://scs.hainanu.edu.cn/ | 邮箱:scscs@hainanu.edu.cn | 电话:0898-66259127; 0898-66257132
 土木建筑工程学院 | http://scea.hainanu.edu.cn | 电话:0898-66279232
 海洋技术与装备学院 | http://smse.hainanu.edu.cn/ | 邮箱:sheny2000@hainanu.edu.cn; 991302@hainanu.edu.cn | 电话:0898-66192572; 0898-66255276
 环境科学与工程学院 | http://sese.hainanu.edu.cn | 电话:0898-66255157
-食品科学与工程学院 | https://hd.hainanu.edu.cn/shipin/
+食品科学与工程学院 | https://foodsci.hainanu.edu.cn | 邮箱:foodsci@hainanu.edu.cn; 992780@hainanu.edu.cn; 992415@hainanu.edu.cn | 电话:0898-66982750; 0898-66982801-; 0898-66192561（
 海洋生物与水产学院 | http://smbf.hainanu.edu.cn | 邮箱:xiesg@hainanu.edu.cn; 993928@hainanu.edu.cn; haiyyb@hainu.edu.cn | 电话:0898-66279184
 空天智能学院 | https://sai.hainanu.edu.cn/ | 邮箱:ktzn@hainanu.edu.cn | 电话:0898-66268297</t>
   </si>
@@ -4133,7 +4133,7 @@
 土木工程与建筑学院 | http://scea.whut.edu.cn/ | 电话:027-87651786
 资源与环境工程学院 | http://sree.whut.edu.cn/
 信息工程学院 | http://wutinfo.whut.edu.cn/
-人工智能学院 | http://csai.whut.edu.cn/
+人工智能学院 | https://ai.whut.edu.cn | 电话:027-87298226; 027-87566996; 027-87687326
 数学与统计学院 | http://maths.whut.edu.cn | 电话:027-87650137（
 物理与力学学院 | http://phymech.whut.edu.cn | 电话:027-87108026（
 化学化工学院 | http://cce.whut.edu.cn/ | 邮箱:hsxy@whut.edu.cn | 电话:027-87749379
@@ -4207,21 +4207,21 @@
     <t>做好处 处长</t>
   </si>
   <si>
-    <t>电气工程与自动化学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=dqxy&amp;type=w
-机械工程及自动化学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=jxxy&amp;type=w
-数学与统计学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=math&amp;type=w
-化工学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=che&amp;type=w
-土木工程学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=civil&amp;type=w
-环境与安全工程学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=es&amp;type=w
-生物科学与工程学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=bio&amp;type=w
-计算机与大数据学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=ccds&amp;type=w
-物理与信息工程学院、微电子学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=wx&amp;type=w
-化学学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=chem&amp;type=w
-建筑与城乡规划学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=jzxy&amp;type=w
-紫金地质与矿业学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=zjxy&amp;type=w
-材料科学与工程学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=cl&amp;type=w
-先进制造学院与海洋学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=xjzz&amp;type=w
-梅努斯国际工程学院 | https://www.fzu.edu.cn/system/resource/link.jsp?bmmc=miec&amp;type=w
+    <t>电气工程与自动化学院 | https://dqxy.fzu.edu.cn/ | 邮箱:dqxy@fzu.edu.cn; zhengx_1976@163.com; feixiongchen@fzu.edu.cn | 电话:0591-22866587; 0591-22866599; 0591-22866588
+机械工程及自动化学院 | https://jxxy.fzu.edu.cn/ | 邮箱:jxxyh@fzu.edu.cn; 819259992@qq.com; renzyrose@126.com | 电话:2024-04-10; 0591-22866262; 0591-22866170
+数学与统计学院 | https://math.fzu.edu.cn/ | 邮箱:yjliu@fzu.edu.cn; hcheng@fzu.edu.cn; jiangfei0591@163.com | 电话:0591-22860369; 0591-22860380; 0591-22860359
+化工学院 | https://che.fzu.edu.cn | 邮箱:syhg@fzu.edu.cn | 电话:0591-22865957; 0591-22865220; 0595-36218102
+土木工程学院 | https://civil.fzu.edu.cn | 电话:0591-22865351; 0591-22865373
+环境与安全工程学院 | https://es.fzu.edu.cn/ | 邮箱:liuwang@fzu.edu.cn; joexu@fzu.edu.cn; 439356896@qq.com | 电话:0591-22866099; 0591-22866356; 0591-22866069
+生物科学与工程学院 | https://bio.fzu.edu.cn | 电话:0591-22866276; 0591-22866277
+计算机与大数据学院 | https://ccds.fzu.edu.cn/ | 邮箱:mchen@fzu.edu.cn
+物理与信息工程学院、微电子学院 | https://wx.fzu.edu.cn | 邮箱:luxiaoqiang@fzu.edu.cn; wjm063@163.com; 1847735879@qq.com | 电话:0591-22865160; 0591-22865127; 0591-22865128
+化学学院 | https://chem.fzu.edu.cn | 邮箱:hxxy@fzu.edu.cn; 821494183@qq.com; zhongyuwu@fzu.edu.cn | 电话:0591-22866234; 0591-22866230; 0591-22866124
+建筑与城乡规划学院 | https://jzxy.fzu.edu.cn | 邮箱:jzxy@fzu.edu.cn | 电话:0591-22887607; 0591-22866383; 0591-22866386
+紫金地质与矿业学院 | https://zjxy.fzu.edu.cn | 邮箱:zjky@fzu.edu.cn | 电话:22865211; 0591-22865218; 0591-22865216
+材料科学与工程学院 | https://cl.fzu.edu.cn | 电话:0591-22866539
+先进制造学院与海洋学院 | https://xjzz.fzu.edu.cn/ | 电话:0595-82660803; 0595-82660810; 82660861（
+梅努斯国际工程学院 | https://miec.fzu.edu.cn | 邮箱:miec@fzu.edu.cn; miec_fzu@163.com; joseph.timoney@mu.ieDr | 电话:0591-22801600; 0591-22801601; 13665029308
 未来技术学院 | https://future.fzu.edu.cn/ | 邮箱:future@fzu.edu.cn | 电话:0591-22863835</t>
   </si>
   <si>

</xml_diff>